<commit_message>
Update: Threat Alert Report - 2026-07-24 23:00
</commit_message>
<xml_diff>
--- a/excel_routes/route_ATZ_JED_threats.xlsx
+++ b/excel_routes/route_ATZ_JED_threats.xlsx
@@ -33,7 +33,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,14 +48,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
-        <bgColor rgb="00FFF3CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
-        <bgColor rgb="00D4EDDA"/>
+        <fgColor rgb="00F8D7DA"/>
+        <bgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -86,9 +80,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -532,7 +523,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>07-JUN-26</t>
+          <t>05-AUG-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -542,30 +533,30 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>EgyptAir MS-643</t>
+          <t>flyadeal F3-778</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>7755</v>
+        <v>7426</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>13289</v>
+        <v>21461</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-5534</v>
+        <v>-14035</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>-16</v>
+        <v>10</v>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -577,7 +568,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>07-JUN-26</t>
+          <t>05-AUG-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -587,30 +578,30 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>EgyptAir MS-641</t>
+          <t>Nile Air NP-227</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>7755</v>
+        <v>10048</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>13289</v>
+        <v>21461</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-5534</v>
+        <v>-11413</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -622,7 +613,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>07-JUN-26</t>
+          <t>05-AUG-26</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -632,30 +623,30 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>EgyptAir MS-665</t>
+          <t>Nile Air NP-127</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>7755</v>
+        <v>10048</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>13289</v>
+        <v>21461</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-5534</v>
+        <v>-11413</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -667,7 +658,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>08-JUN-26</t>
+          <t>05-AUG-26</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -677,30 +668,30 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-127</t>
+          <t>flyadeal F3-754</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4954</v>
+        <v>11863</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>8818</v>
+        <v>21461</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-3864</v>
+        <v>-9598</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>-10</v>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -712,7 +703,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>08-JUN-26</t>
+          <t>05-AUG-26</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -722,17 +713,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>EgyptAir MS-641</t>
+          <t>Saudia SV-6898</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7286</v>
+        <v>11986</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>8818</v>
+        <v>21461</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-1532</v>
+        <v>-9475</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>46</v>
@@ -743,9 +734,9 @@
       <c r="I6" s="2" t="n">
         <v>-16</v>
       </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">

</xml_diff>